<commit_message>
Add Sub Modules to TL Sheet
</commit_message>
<xml_diff>
--- a/Design/TL_Sheet/toplevel.xlsx
+++ b/Design/TL_Sheet/toplevel.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ahmad\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C13B09F-7D0F-4BDA-B657-8D4E65A69BD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D77D9A3-72F0-4373-A393-5FE3D37947AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{2785016E-DC0C-40C4-9ED0-BB5DC1D874D4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{2785016E-DC0C-40C4-9ED0-BB5DC1D874D4}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="toplevel" sheetId="1" r:id="rId1"/>
+    <sheet name="u_mux_1" sheetId="3" r:id="rId2"/>
+    <sheet name="u_mux_2" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="21">
   <si>
     <t>Width</t>
   </si>
@@ -68,6 +70,33 @@
   </si>
   <si>
     <t>2</t>
+  </si>
+  <si>
+    <t>i_sel</t>
+  </si>
+  <si>
+    <t>gen_mux</t>
+  </si>
+  <si>
+    <t>Connection</t>
+  </si>
+  <si>
+    <t>ModuleName</t>
+  </si>
+  <si>
+    <t>dwc_mphy_tx_4l</t>
+  </si>
+  <si>
+    <t>i_data</t>
+  </si>
+  <si>
+    <t>i_parity</t>
+  </si>
+  <si>
+    <t>o_data_mux</t>
+  </si>
+  <si>
+    <t>i_parity[0]</t>
   </si>
 </sst>
 </file>
@@ -83,12 +112,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -103,12 +138,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -425,66 +463,248 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13D79370-5B79-4430-970A-754609A68E6D}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" style="1" customWidth="1"/>
-    <col min="2" max="3" width="15.7109375" style="1" customWidth="1"/>
+    <col min="1" max="2" width="20.7109375" style="1" customWidth="1"/>
+    <col min="3" max="4" width="15.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE1794D1-2CDB-4580-8A12-DCD59719C3BA}">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="20.7109375" style="1" customWidth="1"/>
+    <col min="3" max="4" width="15.7109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>15</v>
+      </c>
       <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="D1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E1B4AAB-E760-465D-B98C-164D2721FDAE}">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="20.7109375" style="1" customWidth="1"/>
+    <col min="3" max="4" width="15.7109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
       <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>5</v>
-      </c>
+      <c r="E2" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>10</v>
-      </c>
+      <c r="E3" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>9</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated TL sheet with more complicated sub modules
</commit_message>
<xml_diff>
--- a/Design/TL_Sheet/toplevel.xlsx
+++ b/Design/TL_Sheet/toplevel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ahmad\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D77D9A3-72F0-4373-A393-5FE3D37947AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FCA152D-85B4-480E-9091-DC937909B16E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{2785016E-DC0C-40C4-9ED0-BB5DC1D874D4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{2785016E-DC0C-40C4-9ED0-BB5DC1D874D4}"/>
   </bookViews>
   <sheets>
     <sheet name="toplevel" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="22">
   <si>
     <t>Width</t>
   </si>
@@ -93,10 +93,13 @@
     <t>i_parity</t>
   </si>
   <si>
-    <t>o_data_mux</t>
-  </si>
-  <si>
-    <t>i_parity[0]</t>
+    <t>data_mux_out</t>
+  </si>
+  <si>
+    <t>parity_data_out</t>
+  </si>
+  <si>
+    <t>scan_rst</t>
   </si>
 </sst>
 </file>
@@ -463,7 +466,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13D79370-5B79-4430-970A-754609A68E6D}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="20.7109375" style="1" customWidth="1"/>
@@ -511,32 +514,32 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>11</v>
@@ -544,12 +547,23 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -560,7 +574,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE1794D1-2CDB-4580-8A12-DCD59719C3BA}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="20.7109375" style="1" customWidth="1"/>
@@ -596,7 +610,7 @@
         <v>4</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>17</v>
@@ -618,15 +632,29 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>19</v>
       </c>
     </row>
@@ -642,7 +670,7 @@
   <cols>
     <col min="1" max="2" width="20.7109375" style="1" customWidth="1"/>
     <col min="3" max="4" width="15.7109375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="5" max="5" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -673,10 +701,10 @@
         <v>4</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -704,7 +732,7 @@
         <v>9</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>